<commit_message>
Removed production files from repository (move to Release Assets); BOM updates
</commit_message>
<xml_diff>
--- a/dvrk-ios-bom.xlsx
+++ b/dvrk-ios-bom.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1DA05DE-9422-4B50-B4DB-773AF6A44EA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98F04BF9-F084-4E89-8AC7-832D8706F9ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="941" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="79">
   <si>
     <t>Notes:</t>
   </si>
@@ -171,9 +171,6 @@
     <t>151-622-009-260-033-ND</t>
   </si>
   <si>
-    <t>Yellow color may be substituted</t>
-  </si>
-  <si>
     <t>490-7198-1-ND</t>
   </si>
   <si>
@@ -201,9 +198,6 @@
     <t>C182375</t>
   </si>
   <si>
-    <t>C2296 (yellow)</t>
-  </si>
-  <si>
     <t>C148025</t>
   </si>
   <si>
@@ -231,9 +225,6 @@
     <t>C1608X7R1C105KT000N</t>
   </si>
   <si>
-    <t>C76617</t>
-  </si>
-  <si>
     <t>TDK</t>
   </si>
   <si>
@@ -268,6 +259,18 @@
   </si>
   <si>
     <t>C4</t>
+  </si>
+  <si>
+    <t>C75749</t>
+  </si>
+  <si>
+    <t>Yellow color may be substituted (JLCPCB #C2296)</t>
+  </si>
+  <si>
+    <t>C2295</t>
+  </si>
+  <si>
+    <t>C59782</t>
   </si>
 </sst>
 </file>
@@ -932,7 +935,7 @@
     <row r="3" spans="1:10" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="10">
-        <v>46062</v>
+        <v>46083</v>
       </c>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
@@ -993,10 +996,10 @@
         <v>7</v>
       </c>
       <c r="I6" s="21" t="s">
+        <v>50</v>
+      </c>
+      <c r="J6" s="21" t="s">
         <v>51</v>
-      </c>
-      <c r="J6" s="21" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="7" spans="1:10" s="32" customFormat="1" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
@@ -1007,28 +1010,28 @@
         <v>1</v>
       </c>
       <c r="C7" s="26" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="D7" s="27" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="E7" s="28" t="s">
         <v>10</v>
       </c>
       <c r="F7" s="29" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="G7" s="30">
         <v>1</v>
       </c>
       <c r="H7" s="31" t="s">
+        <v>62</v>
+      </c>
+      <c r="I7" s="31" t="s">
         <v>64</v>
       </c>
-      <c r="I7" s="31" t="s">
-        <v>67</v>
-      </c>
       <c r="J7" s="31" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
     </row>
     <row r="8" spans="1:10" s="32" customFormat="1" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
@@ -1040,10 +1043,10 @@
         <v>2</v>
       </c>
       <c r="C8" s="26" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="D8" s="27" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E8" s="28" t="s">
         <v>10</v>
@@ -1058,10 +1061,10 @@
         <v>18</v>
       </c>
       <c r="I8" s="27" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="J8" s="27" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="9" spans="1:10" s="32" customFormat="1" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
@@ -1073,10 +1076,10 @@
         <v>1</v>
       </c>
       <c r="C9" s="26" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="D9" s="27" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E9" s="28" t="s">
         <v>10</v>
@@ -1088,13 +1091,13 @@
         <v>1</v>
       </c>
       <c r="H9" s="33" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="I9" s="34" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="J9" s="27" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="10" spans="1:10" s="32" customFormat="1" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
@@ -1123,7 +1126,7 @@
       <c r="H10" s="33"/>
       <c r="I10" s="27"/>
       <c r="J10" s="27" t="s">
-        <v>55</v>
+        <v>77</v>
       </c>
     </row>
     <row r="11" spans="1:10" s="32" customFormat="1" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
@@ -1138,24 +1141,26 @@
         <v>28</v>
       </c>
       <c r="D11" s="27" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="E11" s="28" t="s">
         <v>43</v>
       </c>
       <c r="F11" s="29" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="G11" s="30">
         <v>1</v>
       </c>
       <c r="H11" s="34" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="I11" s="27" t="s">
         <v>44</v>
       </c>
-      <c r="J11" s="27"/>
+      <c r="J11" s="27" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="12" spans="1:10" s="32" customFormat="1" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="24">
@@ -1185,7 +1190,7 @@
         <v>20</v>
       </c>
       <c r="J12" s="27" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="13" spans="1:10" s="32" customFormat="1" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
@@ -1200,25 +1205,25 @@
         <v>30</v>
       </c>
       <c r="D13" s="27" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E13" s="28" t="s">
         <v>10</v>
       </c>
       <c r="F13" s="29" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="G13" s="30">
         <v>1</v>
       </c>
       <c r="H13" s="33" t="s">
+        <v>59</v>
+      </c>
+      <c r="I13" s="27" t="s">
         <v>61</v>
       </c>
-      <c r="I13" s="27" t="s">
-        <v>63</v>
-      </c>
       <c r="J13" s="27" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="14" spans="1:10" s="32" customFormat="1" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
@@ -1233,7 +1238,7 @@
         <v>31</v>
       </c>
       <c r="D14" s="27" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="E14" s="28" t="s">
         <v>10</v>
@@ -1247,7 +1252,7 @@
       <c r="H14" s="33"/>
       <c r="I14" s="27"/>
       <c r="J14" s="27" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="15" spans="1:10" s="32" customFormat="1" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
@@ -1278,7 +1283,7 @@
         <v>42</v>
       </c>
       <c r="J15" s="27" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="16" spans="1:10" s="32" customFormat="1" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
@@ -1309,7 +1314,7 @@
         <v>40</v>
       </c>
       <c r="J16" s="27" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="17" spans="1:10" s="32" customFormat="1" ht="16.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -1322,7 +1327,7 @@
       </c>
       <c r="C17" s="38"/>
       <c r="D17" s="39" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="E17" s="40"/>
       <c r="F17" s="39"/>
@@ -1407,7 +1412,7 @@
         <v>2</v>
       </c>
       <c r="C23" s="34" t="s">
-        <v>45</v>
+        <v>76</v>
       </c>
       <c r="D23" s="34"/>
       <c r="E23" s="43"/>

</xml_diff>